<commit_message>
Validate Identity's spec/design note, add 04_01b as its own manual gate
Adds the validated behavior spec and approved design note for the Identity
slice. Amends the master migration plan so design-note approval is a formal
gate (04_01b) alongside spec approval (03_02) and code review (04_05),
mirroring the same "catch it on paper, before code exists" logic - the
tracker's own status legend already implied this review step existed, but
the plan's table/diagram never named it. Updates the tracker and READMEs
to match, and adds HTML summaries of the migration plan for demo walkthroughs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/migration_support/migration-tracker.xlsx
+++ b/migration_support/migration-tracker.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Migration Tracker" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,13 +12,15 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Migration Tracker'!$A$1:$I$6</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -31,10 +32,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -46,8 +49,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,23 +64,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -85,9 +89,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -451,7 +458,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -464,7 +471,7 @@
     <col width="55" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="27.6" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Order</t>
@@ -511,7 +518,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="27.6" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -530,15 +537,25 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>Code In Progress</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>migration_support/03_01_java_api_slice_behaviour_doc/01-identity-spec.md</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>muthuramanmca@gmail.com</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>46236</v>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Foundational - no dependencies; migrate first</t>
+          <t>Foundational - no dependencies; migrate first. Spec validated in chat. Design note: migration_support/04_01_net_slice_design_note/01-identity-design.md. 04_02 (register/login/me + outbox) implemented and building green; next is 04_03 (unit tests, from the spec) and 04_04 (Java/.NET compare), then 04_05 (code review, manual gate).</t>
         </is>
       </c>
     </row>
@@ -564,16 +581,16 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>No dependencies on other slices</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="27.6" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -595,16 +612,16 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Calls FlightService.findOrThrow directly; needs both prior slices in place to build/test against</t>
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="41.4" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -626,16 +643,16 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Account auto-created via PassengerRegisteredEvent (Identity); miles awarded via BookingPaidEvent (Booking) -- both event-mediated, not direct calls</t>
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="27.6" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -657,9 +674,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Triggered by BookingCreatedEvent and BookingPaidEvent (Booking) -- event-mediated, not a direct call</t>
@@ -684,7 +701,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
@@ -714,7 +731,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="27.6" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Queued for Drafting</t>

</xml_diff>